<commit_message>
Template Tradicional atualizado e formato de célula dos condomínios
- Novo template Tradicional (sem a coluna Ampla); bloco de Plano de Vida
  duplicado removido de novo, mesclas da linha 1 refeitas.
- preencher_massa: formato por ramo. Condomínios seguem a linha de
  exemplo do template: marcado 'Sim', desmarcado 'Não', não contratado
  vazio, valores como número. Empresarial/residencial sem mudança.
- Docs: catalogo_condominio, lmi_condominio_tradicional e SKILL.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETeciituSBa5wphWUasW8C
</commit_message>
<xml_diff>
--- a/.claude/skills/gerador-massas-seguros/templates/template_condominio_tradicional.xlsx
+++ b/.claude/skills/gerador-massas-seguros/templates/template_condominio_tradicional.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Auxiliar" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -15,8 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="9">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="00000000000000"/>
+    <numFmt numFmtId="165" formatCode="00000000"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -33,16 +38,19 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <color rgb="FFF3F3F3"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
@@ -65,10 +73,23 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -152,6 +173,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -225,10 +252,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -243,9 +271,6 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -267,6 +292,32 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -287,9 +338,11 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -684,172 +737,170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE10"/>
+  <dimension ref="A1:BD11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.85546875" bestFit="1" customWidth="1" style="18" min="1" max="1"/>
-    <col width="18.42578125" bestFit="1" customWidth="1" style="18" min="2" max="2"/>
-    <col width="12" bestFit="1" customWidth="1" style="18" min="3" max="3"/>
-    <col width="8" bestFit="1" customWidth="1" style="18" min="4" max="4"/>
-    <col width="63.5703125" customWidth="1" style="18" min="5" max="5"/>
-    <col width="30.5703125" customWidth="1" style="18" min="6" max="6"/>
-    <col width="26.5703125" customWidth="1" style="18" min="7" max="7"/>
-    <col width="44.140625" customWidth="1" style="18" min="8" max="8"/>
-    <col width="33" bestFit="1" customWidth="1" style="18" min="9" max="9"/>
-    <col width="42.140625" bestFit="1" customWidth="1" style="18" min="10" max="10"/>
-    <col width="60.42578125" bestFit="1" customWidth="1" style="18" min="11" max="11"/>
-    <col width="27.5703125" bestFit="1" customWidth="1" style="18" min="12" max="12"/>
-    <col width="29.42578125" bestFit="1" customWidth="1" style="18" min="13" max="13"/>
-    <col width="76.28515625" bestFit="1" customWidth="1" style="18" min="14" max="14"/>
-    <col width="77.28515625" bestFit="1" customWidth="1" style="18" min="15" max="15"/>
-    <col width="78.28515625" bestFit="1" customWidth="1" style="18" min="16" max="16"/>
-    <col width="82.7109375" bestFit="1" customWidth="1" style="18" min="17" max="17"/>
-    <col width="76.85546875" bestFit="1" customWidth="1" style="18" min="18" max="18"/>
-    <col width="82.7109375" bestFit="1" customWidth="1" style="18" min="19" max="19"/>
-    <col width="41.7109375" bestFit="1" customWidth="1" style="18" min="20" max="20"/>
-    <col width="40.7109375" bestFit="1" customWidth="1" style="18" min="21" max="21"/>
-    <col width="41.7109375" bestFit="1" customWidth="1" style="18" min="22" max="23"/>
-    <col width="13" customWidth="1" style="18" min="23" max="23"/>
-    <col width="47.7109375" bestFit="1" customWidth="1" style="18" min="24" max="24"/>
-    <col width="53.5703125" bestFit="1" customWidth="1" style="18" min="25" max="25"/>
-    <col width="69.7109375" bestFit="1" customWidth="1" style="18" min="26" max="26"/>
-    <col width="79.7109375" bestFit="1" customWidth="1" style="18" min="27" max="27"/>
-    <col width="62" bestFit="1" customWidth="1" style="18" min="28" max="28"/>
-    <col width="32.5703125" bestFit="1" customWidth="1" style="18" min="29" max="29"/>
-    <col width="40.28515625" bestFit="1" customWidth="1" style="18" min="30" max="30"/>
-    <col width="36" bestFit="1" customWidth="1" style="18" min="31" max="31"/>
-    <col width="76.140625" bestFit="1" customWidth="1" style="18" min="32" max="32"/>
-    <col width="53.140625" bestFit="1" customWidth="1" style="18" min="33" max="33"/>
-    <col width="53.42578125" bestFit="1" customWidth="1" style="18" min="34" max="34"/>
-    <col width="53.28515625" bestFit="1" customWidth="1" style="18" min="35" max="35"/>
-    <col width="52.42578125" bestFit="1" customWidth="1" style="18" min="36" max="36"/>
-    <col width="60.5703125" bestFit="1" customWidth="1" style="18" min="37" max="37"/>
-    <col width="60.42578125" bestFit="1" customWidth="1" style="18" min="38" max="38"/>
-    <col width="37.28515625" bestFit="1" customWidth="1" style="18" min="39" max="39"/>
-    <col width="55.140625" bestFit="1" customWidth="1" style="18" min="40" max="40"/>
-    <col width="101.42578125" bestFit="1" customWidth="1" style="18" min="41" max="41"/>
-    <col width="108.7109375" bestFit="1" customWidth="1" style="18" min="42" max="42"/>
-    <col width="49.85546875" bestFit="1" customWidth="1" style="18" min="43" max="43"/>
-    <col width="37.5703125" bestFit="1" customWidth="1" style="18" min="44" max="44"/>
-    <col width="68.5703125" bestFit="1" customWidth="1" style="18" min="45" max="45"/>
-    <col width="51.5703125" bestFit="1" customWidth="1" style="18" min="46" max="46"/>
-    <col width="46.42578125" bestFit="1" customWidth="1" style="18" min="47" max="47"/>
-    <col width="81.28515625" bestFit="1" customWidth="1" style="18" min="48" max="48"/>
-    <col width="27.85546875" bestFit="1" customWidth="1" style="18" min="49" max="49"/>
-    <col width="27.28515625" bestFit="1" customWidth="1" style="18" min="50" max="50"/>
-    <col width="21.5703125" bestFit="1" customWidth="1" style="18" min="51" max="51"/>
-    <col width="70.85546875" bestFit="1" customWidth="1" style="18" min="52" max="52"/>
-    <col width="56.5703125" bestFit="1" customWidth="1" style="18" min="53" max="53"/>
-    <col width="69.5703125" bestFit="1" customWidth="1" style="18" min="54" max="54"/>
-    <col width="34" bestFit="1" customWidth="1" style="18" min="55" max="55"/>
-    <col width="34.85546875" bestFit="1" customWidth="1" style="18" min="56" max="56"/>
-    <col width="35.140625" bestFit="1" customWidth="1" style="18" min="57" max="57"/>
-    <col width="27.28515625" bestFit="1" customWidth="1" style="18" min="58" max="58"/>
-    <col width="21.5703125" bestFit="1" customWidth="1" style="18" min="59" max="59"/>
-    <col width="70.85546875" bestFit="1" customWidth="1" style="18" min="60" max="60"/>
-    <col width="56.5703125" bestFit="1" customWidth="1" style="18" min="61" max="61"/>
-    <col width="69.5703125" bestFit="1" customWidth="1" style="18" min="62" max="62"/>
-    <col width="34" bestFit="1" customWidth="1" style="18" min="63" max="63"/>
-    <col width="34.85546875" bestFit="1" customWidth="1" style="18" min="64" max="64"/>
-    <col width="35.140625" bestFit="1" customWidth="1" style="18" min="65" max="65"/>
+    <col width="10.85546875" bestFit="1" customWidth="1" style="27" min="1" max="1"/>
+    <col width="18.42578125" bestFit="1" customWidth="1" style="27" min="2" max="2"/>
+    <col width="15.140625" bestFit="1" customWidth="1" style="27" min="3" max="3"/>
+    <col width="9" bestFit="1" customWidth="1" style="27" min="4" max="4"/>
+    <col width="63.5703125" customWidth="1" style="27" min="5" max="5"/>
+    <col width="30.5703125" customWidth="1" style="27" min="6" max="6"/>
+    <col width="26.5703125" customWidth="1" style="27" min="7" max="7"/>
+    <col width="44.140625" customWidth="1" style="27" min="8" max="8"/>
+    <col width="33" bestFit="1" customWidth="1" style="27" min="9" max="9"/>
+    <col width="45.85546875" bestFit="1" customWidth="1" style="27" min="10" max="10"/>
+    <col width="60.42578125" bestFit="1" customWidth="1" style="27" min="11" max="11"/>
+    <col width="27.5703125" bestFit="1" customWidth="1" style="27" min="12" max="12"/>
+    <col width="29.42578125" bestFit="1" customWidth="1" style="27" min="13" max="13"/>
+    <col width="76.28515625" bestFit="1" customWidth="1" style="27" min="14" max="14"/>
+    <col width="77.28515625" bestFit="1" customWidth="1" style="27" min="15" max="15"/>
+    <col width="78.28515625" bestFit="1" customWidth="1" style="27" min="16" max="16"/>
+    <col width="82.7109375" bestFit="1" customWidth="1" style="27" min="17" max="17"/>
+    <col width="76.85546875" bestFit="1" customWidth="1" style="27" min="18" max="18"/>
+    <col width="82.7109375" bestFit="1" customWidth="1" style="27" min="19" max="19"/>
+    <col width="41.7109375" bestFit="1" customWidth="1" style="27" min="20" max="20"/>
+    <col width="40.7109375" bestFit="1" customWidth="1" style="27" min="21" max="21"/>
+    <col width="41.7109375" bestFit="1" customWidth="1" style="27" min="22" max="23"/>
+    <col width="13" customWidth="1" style="27" min="23" max="23"/>
+    <col width="47.7109375" bestFit="1" customWidth="1" style="27" min="24" max="24"/>
+    <col width="53.5703125" bestFit="1" customWidth="1" style="27" min="25" max="25"/>
+    <col width="69.7109375" bestFit="1" customWidth="1" style="27" min="26" max="26"/>
+    <col width="79.7109375" bestFit="1" customWidth="1" style="27" min="27" max="27"/>
+    <col width="62" bestFit="1" customWidth="1" style="27" min="28" max="28"/>
+    <col width="32.5703125" bestFit="1" customWidth="1" style="27" min="29" max="29"/>
+    <col width="40.28515625" bestFit="1" customWidth="1" style="27" min="30" max="30"/>
+    <col width="36" bestFit="1" customWidth="1" style="27" min="31" max="31"/>
+    <col width="76.140625" bestFit="1" customWidth="1" style="27" min="32" max="32"/>
+    <col width="53.140625" bestFit="1" customWidth="1" style="27" min="33" max="33"/>
+    <col width="53.42578125" bestFit="1" customWidth="1" style="27" min="34" max="34"/>
+    <col width="53.28515625" bestFit="1" customWidth="1" style="27" min="35" max="35"/>
+    <col width="52.42578125" bestFit="1" customWidth="1" style="27" min="36" max="36"/>
+    <col width="60.5703125" bestFit="1" customWidth="1" style="27" min="37" max="37"/>
+    <col width="60.42578125" bestFit="1" customWidth="1" style="27" min="38" max="38"/>
+    <col width="37.28515625" bestFit="1" customWidth="1" style="27" min="39" max="39"/>
+    <col width="55.140625" bestFit="1" customWidth="1" style="27" min="40" max="40"/>
+    <col width="101.42578125" bestFit="1" customWidth="1" style="27" min="41" max="41"/>
+    <col width="108.7109375" bestFit="1" customWidth="1" style="27" min="42" max="42"/>
+    <col width="49.85546875" bestFit="1" customWidth="1" style="27" min="43" max="43"/>
+    <col width="37.5703125" bestFit="1" customWidth="1" style="27" min="44" max="44"/>
+    <col width="68.5703125" bestFit="1" customWidth="1" style="27" min="45" max="45"/>
+    <col width="51.5703125" bestFit="1" customWidth="1" style="27" min="46" max="46"/>
+    <col width="46.42578125" bestFit="1" customWidth="1" style="27" min="47" max="47"/>
+    <col width="81.28515625" bestFit="1" customWidth="1" style="27" min="48" max="48"/>
+    <col width="27.28515625" bestFit="1" customWidth="1" style="27" min="49" max="49"/>
+    <col width="21.5703125" bestFit="1" customWidth="1" style="27" min="50" max="50"/>
+    <col width="70.85546875" bestFit="1" customWidth="1" style="27" min="51" max="51"/>
+    <col width="56.5703125" bestFit="1" customWidth="1" style="27" min="52" max="52"/>
+    <col width="69.5703125" bestFit="1" customWidth="1" style="27" min="53" max="53"/>
+    <col width="34" bestFit="1" customWidth="1" style="27" min="54" max="54"/>
+    <col width="34.85546875" bestFit="1" customWidth="1" style="27" min="55" max="55"/>
+    <col width="35.140625" bestFit="1" customWidth="1" style="27" min="56" max="56"/>
+    <col width="27.28515625" bestFit="1" customWidth="1" style="27" min="57" max="57"/>
+    <col width="21.5703125" bestFit="1" customWidth="1" style="27" min="58" max="58"/>
+    <col width="70.85546875" bestFit="1" customWidth="1" style="27" min="59" max="59"/>
+    <col width="56.5703125" bestFit="1" customWidth="1" style="27" min="60" max="60"/>
+    <col width="69.5703125" bestFit="1" customWidth="1" style="27" min="61" max="61"/>
+    <col width="34" bestFit="1" customWidth="1" style="27" min="62" max="62"/>
+    <col width="34.85546875" bestFit="1" customWidth="1" style="27" min="63" max="63"/>
+    <col width="35.140625" bestFit="1" customWidth="1" style="27" min="64" max="64"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="n"/>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>Dados CORRETOR</t>
         </is>
       </c>
-      <c r="D1" s="19" t="inlineStr">
+      <c r="D1" s="28" t="inlineStr">
         <is>
           <t>Caracteristaca do Risco</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Questionario 1</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>Questionario 2</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Questionario 3</t>
         </is>
       </c>
-      <c r="M1" s="11" t="inlineStr">
+      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>Questionario 4</t>
         </is>
       </c>
-      <c r="N1" s="20" t="inlineStr">
+      <c r="N1" s="29" t="inlineStr">
         <is>
           <t>Questionario 5 - Quantidade de Pavimentos</t>
         </is>
       </c>
-      <c r="O1" s="23" t="n"/>
-      <c r="P1" s="23" t="n"/>
-      <c r="Q1" s="23" t="n"/>
-      <c r="R1" s="23" t="n"/>
-      <c r="S1" s="8" t="inlineStr">
+      <c r="O1" s="32" t="n"/>
+      <c r="P1" s="32" t="n"/>
+      <c r="Q1" s="32" t="n"/>
+      <c r="R1" s="32" t="n"/>
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>Questionario - 6</t>
         </is>
       </c>
-      <c r="T1" s="21" t="inlineStr">
+      <c r="T1" s="30" t="inlineStr">
         <is>
           <t>Questionario - 7 QUAL IDADE DO CONDOMINIO</t>
         </is>
       </c>
-      <c r="U1" s="23" t="n"/>
-      <c r="V1" s="23" t="n"/>
-      <c r="W1" s="23" t="n"/>
-      <c r="X1" s="23" t="n"/>
-      <c r="Y1" s="22" t="inlineStr">
+      <c r="U1" s="32" t="n"/>
+      <c r="V1" s="32" t="n"/>
+      <c r="W1" s="32" t="n"/>
+      <c r="X1" s="32" t="n"/>
+      <c r="Y1" s="31" t="inlineStr">
         <is>
           <t>Coberturas</t>
         </is>
       </c>
-      <c r="Z1" s="23" t="n"/>
-      <c r="AA1" s="23" t="n"/>
-      <c r="AB1" s="23" t="n"/>
-      <c r="AC1" s="23" t="n"/>
-      <c r="AD1" s="23" t="n"/>
-      <c r="AE1" s="23" t="n"/>
-      <c r="AF1" s="23" t="n"/>
-      <c r="AG1" s="23" t="n"/>
-      <c r="AH1" s="23" t="n"/>
-      <c r="AI1" s="23" t="n"/>
-      <c r="AJ1" s="23" t="n"/>
-      <c r="AK1" s="23" t="n"/>
-      <c r="AL1" s="23" t="n"/>
-      <c r="AM1" s="23" t="n"/>
-      <c r="AN1" s="23" t="n"/>
-      <c r="AO1" s="23" t="n"/>
-      <c r="AP1" s="23" t="n"/>
-      <c r="AQ1" s="23" t="n"/>
-      <c r="AR1" s="23" t="n"/>
-      <c r="AS1" s="23" t="n"/>
-      <c r="AT1" s="23" t="n"/>
-      <c r="AU1" s="23" t="n"/>
-      <c r="AV1" s="23" t="n"/>
-      <c r="AW1" s="23" t="n"/>
-      <c r="AX1" s="16" t="inlineStr">
+      <c r="Z1" s="32" t="n"/>
+      <c r="AA1" s="32" t="n"/>
+      <c r="AB1" s="32" t="n"/>
+      <c r="AC1" s="32" t="n"/>
+      <c r="AD1" s="32" t="n"/>
+      <c r="AE1" s="32" t="n"/>
+      <c r="AF1" s="32" t="n"/>
+      <c r="AG1" s="32" t="n"/>
+      <c r="AH1" s="32" t="n"/>
+      <c r="AI1" s="32" t="n"/>
+      <c r="AJ1" s="32" t="n"/>
+      <c r="AK1" s="32" t="n"/>
+      <c r="AL1" s="32" t="n"/>
+      <c r="AM1" s="32" t="n"/>
+      <c r="AN1" s="32" t="n"/>
+      <c r="AO1" s="32" t="n"/>
+      <c r="AP1" s="32" t="n"/>
+      <c r="AQ1" s="32" t="n"/>
+      <c r="AR1" s="32" t="n"/>
+      <c r="AS1" s="32" t="n"/>
+      <c r="AT1" s="32" t="n"/>
+      <c r="AU1" s="32" t="n"/>
+      <c r="AV1" s="32" t="n"/>
+      <c r="AW1" s="25" t="inlineStr">
         <is>
           <t>Coberturas Plano de Vida</t>
         </is>
       </c>
-      <c r="AY1" s="23" t="n"/>
-      <c r="AZ1" s="23" t="n"/>
-      <c r="BA1" s="23" t="n"/>
-      <c r="BB1" s="23" t="n"/>
-      <c r="BC1" s="23" t="n"/>
-      <c r="BD1" s="23" t="n"/>
-      <c r="BE1" s="23" t="n"/>
+      <c r="AX1" s="32" t="n"/>
+      <c r="AY1" s="32" t="n"/>
+      <c r="AZ1" s="32" t="n"/>
+      <c r="BA1" s="32" t="n"/>
+      <c r="BB1" s="32" t="n"/>
+      <c r="BC1" s="32" t="n"/>
+      <c r="BD1" s="32" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1092,53 +1143,48 @@
           <t>TXT "Vendaval, Furacão, Ciclone, Tornado, Granizo e Impacto de Veículos" Valor da Cobertura</t>
         </is>
       </c>
-      <c r="AW2" s="5" t="inlineStr">
-        <is>
-          <t>TXT "Ampla" Valor da Cobertura</t>
-        </is>
-      </c>
-      <c r="AX2" s="12" t="inlineStr">
+      <c r="AW2" s="11" t="inlineStr">
         <is>
           <t>TXT "Morte" Valor da Cobertura</t>
         </is>
       </c>
-      <c r="AY2" s="12" t="inlineStr">
+      <c r="AX2" s="11" t="inlineStr">
         <is>
           <t>TXT " Qt de vidas" Morte</t>
         </is>
       </c>
-      <c r="AZ2" s="12" t="inlineStr">
+      <c r="AY2" s="11" t="inlineStr">
         <is>
           <t>TXT "Invalidez Permanente Total Ou Parcial Por Acidente (ipa)" Valor da Cobertura</t>
         </is>
       </c>
-      <c r="BA2" s="12" t="inlineStr">
+      <c r="AZ2" s="11" t="inlineStr">
         <is>
           <t>TXT "Indenização Especial Por Acidente (iea)" Valor da Cobertura</t>
         </is>
       </c>
-      <c r="BB2" s="12" t="inlineStr">
+      <c r="BA2" s="11" t="inlineStr">
         <is>
           <t>TXT "Invalidez Funcional Permanente Total Por Doença (ifpd)" Valor da Cobertura</t>
         </is>
       </c>
-      <c r="BC2" s="12" t="inlineStr">
+      <c r="BB2" s="11" t="inlineStr">
         <is>
           <t>TXT "Valor da Cobertura" Cesta Básica</t>
         </is>
       </c>
-      <c r="BD2" s="12" t="inlineStr">
+      <c r="BC2" s="11" t="inlineStr">
         <is>
           <t>TXT "Morte Cônjuge" Valor da Cobertura</t>
         </is>
       </c>
-      <c r="BE2" s="12" t="inlineStr">
+      <c r="BD2" s="11" t="inlineStr">
         <is>
           <t>TXT "Auxílio Funeral" Valor da Cobertura</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20.25" customHeight="1" s="18">
+    <row r="3" ht="20.25" customHeight="1" s="27">
       <c r="A3" t="inlineStr">
         <is>
           <t>Corretor</t>
@@ -1149,163 +1195,886 @@
           <t>COI</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
-        <v>42907871865</v>
-      </c>
-      <c r="D3" s="6" t="n">
+      <c r="C3" s="18" t="n">
+        <v>72066486000171</v>
+      </c>
+      <c r="D3" s="19" t="n">
         <v>6417050</v>
       </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio Comercial - Vertical</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Condomínio Exclusivamente Residencial - Horizontal</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>Superior / Sólida</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="12" t="inlineStr">
         <is>
           <t>Prédio e Conteúdo</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="H3" s="12" t="inlineStr">
         <is>
           <t>Assistência Condomínio Plano Intermediário</t>
         </is>
       </c>
-      <c r="J3" s="15" t="inlineStr">
+      <c r="I3" s="33" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="L3" s="14" t="inlineStr">
+      <c r="K3" s="13" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="R3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="S3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="U3" s="13" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="V3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="W3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="X3" s="13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="Y3" s="33" t="n">
+        <v>10000</v>
+      </c>
+      <c r="Z3" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AA3" s="33" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="AB3" s="33" t="n"/>
+      <c r="AC3" s="33" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AD3" s="33" t="n">
+        <v>2000</v>
+      </c>
+      <c r="AE3" s="33" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AF3" s="33" t="n">
+        <v>15000</v>
+      </c>
+      <c r="AG3" s="33" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AH3" s="33" t="n">
+        <v>35000</v>
+      </c>
+      <c r="AI3" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AJ3" s="33" t="n">
+        <v>75000</v>
+      </c>
+      <c r="AK3" s="33" t="n">
+        <v>35000</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM3" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AN3" s="33" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AO3" s="33" t="n">
+        <v>20000</v>
+      </c>
+      <c r="AP3" s="33" t="n"/>
+      <c r="AQ3" s="33" t="n">
+        <v>20000</v>
+      </c>
+      <c r="AR3" s="33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AS3" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AT3" s="33" t="n">
+        <v>20000</v>
+      </c>
+      <c r="AU3" s="33" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AV3" s="33" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AW3" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AX3" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="AY3" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AZ3" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="BA3" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="BB3" s="33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="BC3" s="33" t="n">
+        <v>2500</v>
+      </c>
+      <c r="BD3" s="33" t="n">
+        <v>3000</v>
+      </c>
     </row>
-    <row r="4" ht="13.5" customHeight="1" s="18">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Operações</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Espaco informatica</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio de Consultórios</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>Mista</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>Assistência Condomínio Plano Básico</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>6 ou mais</t>
-        </is>
-      </c>
+    <row r="4" ht="13.5" customHeight="1" s="27">
+      <c r="C4" s="18" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="12" t="n"/>
+      <c r="F4" s="12" t="n"/>
+      <c r="G4" s="12" t="n"/>
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="33" t="n"/>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="13" t="n"/>
+      <c r="L4" s="13" t="n"/>
+      <c r="N4" s="13" t="n"/>
+      <c r="O4" s="13" t="n"/>
+      <c r="P4" s="13" t="n"/>
+      <c r="Q4" s="13" t="n"/>
+      <c r="R4" s="13" t="n"/>
+      <c r="S4" s="13" t="n"/>
+      <c r="T4" s="13" t="n"/>
+      <c r="U4" s="13" t="n"/>
+      <c r="V4" s="13" t="n"/>
+      <c r="W4" s="13" t="n"/>
+      <c r="X4" s="13" t="n"/>
+      <c r="Y4" s="33" t="n"/>
+      <c r="Z4" s="33" t="n"/>
+      <c r="AA4" s="33" t="n"/>
+      <c r="AB4" s="33" t="n"/>
+      <c r="AC4" s="33" t="n"/>
+      <c r="AD4" s="33" t="n"/>
+      <c r="AE4" s="33" t="n"/>
+      <c r="AF4" s="33" t="n"/>
+      <c r="AG4" s="33" t="n"/>
+      <c r="AH4" s="33" t="n"/>
+      <c r="AI4" s="24" t="n"/>
+      <c r="AJ4" s="33" t="n"/>
+      <c r="AK4" s="33" t="n"/>
+      <c r="AM4" s="33" t="n"/>
+      <c r="AN4" s="33" t="n"/>
+      <c r="AO4" s="33" t="n"/>
+      <c r="AP4" s="33" t="n"/>
+      <c r="AQ4" s="33" t="n"/>
+      <c r="AR4" s="33" t="n"/>
+      <c r="AS4" s="33" t="n"/>
+      <c r="AT4" s="33" t="n"/>
+      <c r="AU4" s="33" t="n"/>
+      <c r="AV4" s="33" t="n"/>
+      <c r="AW4" s="33" t="n"/>
+      <c r="AY4" s="33" t="n"/>
+      <c r="AZ4" s="33" t="n"/>
+      <c r="BA4" s="33" t="n"/>
+      <c r="BB4" s="33" t="n"/>
+      <c r="BC4" s="33" t="n"/>
+      <c r="BD4" s="33" t="n"/>
     </row>
-    <row r="5" ht="15" customHeight="1" s="18">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Subscrição</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Sicredi</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio de Escritórios</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>Não Contratado</t>
-        </is>
-      </c>
+    <row r="5" ht="15" customHeight="1" s="27">
+      <c r="C5" s="18" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="12" t="n"/>
+      <c r="F5" s="12" t="n"/>
+      <c r="G5" s="12" t="n"/>
+      <c r="H5" s="12" t="n"/>
+      <c r="I5" s="33" t="n"/>
+      <c r="J5" s="14" t="n"/>
+      <c r="K5" s="13" t="n"/>
+      <c r="L5" s="13" t="n"/>
+      <c r="N5" s="13" t="n"/>
+      <c r="O5" s="13" t="n"/>
+      <c r="P5" s="13" t="n"/>
+      <c r="Q5" s="13" t="n"/>
+      <c r="R5" s="13" t="n"/>
+      <c r="S5" s="13" t="n"/>
+      <c r="T5" s="13" t="n"/>
+      <c r="U5" s="13" t="n"/>
+      <c r="V5" s="13" t="n"/>
+      <c r="W5" s="13" t="n"/>
+      <c r="X5" s="13" t="n"/>
+      <c r="Y5" s="33" t="n"/>
+      <c r="Z5" s="33" t="n"/>
+      <c r="AA5" s="33" t="n"/>
+      <c r="AB5" s="33" t="n"/>
+      <c r="AC5" s="33" t="n"/>
+      <c r="AD5" s="33" t="n"/>
+      <c r="AE5" s="33" t="n"/>
+      <c r="AF5" s="33" t="n"/>
+      <c r="AG5" s="33" t="n"/>
+      <c r="AH5" s="33" t="n"/>
+      <c r="AI5" s="24" t="n"/>
+      <c r="AJ5" s="33" t="n"/>
+      <c r="AK5" s="33" t="n"/>
+      <c r="AM5" s="33" t="n"/>
+      <c r="AN5" s="33" t="n"/>
+      <c r="AO5" s="33" t="n"/>
+      <c r="AP5" s="33" t="n"/>
+      <c r="AQ5" s="33" t="n"/>
+      <c r="AR5" s="33" t="n"/>
+      <c r="AS5" s="33" t="n"/>
+      <c r="AT5" s="33" t="n"/>
+      <c r="AU5" s="33" t="n"/>
+      <c r="AV5" s="33" t="n"/>
+      <c r="AW5" s="33" t="n"/>
+      <c r="AY5" s="33" t="n"/>
+      <c r="AZ5" s="33" t="n"/>
+      <c r="BA5" s="33" t="n"/>
+      <c r="BB5" s="33" t="n"/>
+      <c r="BC5" s="33" t="n"/>
+      <c r="BD5" s="33" t="n"/>
     </row>
-    <row r="6" ht="15.75" customHeight="1" s="18">
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio Exclusivamente Residencial - Horizontal</t>
-        </is>
-      </c>
+    <row r="6" ht="15.75" customHeight="1" s="27">
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="12" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="33" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="13" t="n"/>
+      <c r="L6" s="13" t="n"/>
+      <c r="N6" s="13" t="n"/>
+      <c r="O6" s="13" t="n"/>
+      <c r="P6" s="13" t="n"/>
+      <c r="Q6" s="13" t="n"/>
+      <c r="R6" s="13" t="n"/>
+      <c r="S6" s="13" t="n"/>
+      <c r="T6" s="13" t="n"/>
+      <c r="U6" s="13" t="n"/>
+      <c r="V6" s="13" t="n"/>
+      <c r="W6" s="13" t="n"/>
+      <c r="X6" s="13" t="n"/>
+      <c r="Y6" s="33" t="n"/>
+      <c r="Z6" s="33" t="n"/>
+      <c r="AA6" s="33" t="n"/>
+      <c r="AB6" s="33" t="n"/>
+      <c r="AC6" s="33" t="n"/>
+      <c r="AD6" s="33" t="n"/>
+      <c r="AE6" s="33" t="n"/>
+      <c r="AF6" s="33" t="n"/>
+      <c r="AG6" s="33" t="n"/>
+      <c r="AH6" s="33" t="n"/>
+      <c r="AI6" s="24" t="n"/>
+      <c r="AJ6" s="33" t="n"/>
+      <c r="AK6" s="33" t="n"/>
+      <c r="AM6" s="33" t="n"/>
+      <c r="AN6" s="33" t="n"/>
+      <c r="AO6" s="33" t="n"/>
+      <c r="AP6" s="33" t="n"/>
+      <c r="AQ6" s="33" t="n"/>
+      <c r="AR6" s="33" t="n"/>
+      <c r="AS6" s="33" t="n"/>
+      <c r="AT6" s="33" t="n"/>
+      <c r="AU6" s="33" t="n"/>
+      <c r="AV6" s="33" t="n"/>
+      <c r="AW6" s="33" t="n"/>
+      <c r="AY6" s="33" t="n"/>
+      <c r="AZ6" s="33" t="n"/>
+      <c r="BA6" s="33" t="n"/>
+      <c r="BB6" s="33" t="n"/>
+      <c r="BC6" s="33" t="n"/>
+      <c r="BD6" s="33" t="n"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1" s="18">
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio Exclusivamente Residencial - Vertical</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="n"/>
+    <row r="7" ht="15.75" customHeight="1" s="27">
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="33" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="13" t="n"/>
+      <c r="L7" s="13" t="n"/>
+      <c r="N7" s="13" t="n"/>
+      <c r="O7" s="13" t="n"/>
+      <c r="P7" s="13" t="n"/>
+      <c r="Q7" s="13" t="n"/>
+      <c r="R7" s="13" t="n"/>
+      <c r="S7" s="13" t="n"/>
+      <c r="T7" s="13" t="n"/>
+      <c r="U7" s="13" t="n"/>
+      <c r="V7" s="13" t="n"/>
+      <c r="W7" s="13" t="n"/>
+      <c r="X7" s="13" t="n"/>
+      <c r="Y7" s="33" t="n"/>
+      <c r="Z7" s="33" t="n"/>
+      <c r="AA7" s="33" t="n"/>
+      <c r="AB7" s="33" t="n"/>
+      <c r="AC7" s="33" t="n"/>
+      <c r="AD7" s="33" t="n"/>
+      <c r="AE7" s="33" t="n"/>
+      <c r="AF7" s="33" t="n"/>
+      <c r="AG7" s="33" t="n"/>
+      <c r="AH7" s="33" t="n"/>
+      <c r="AI7" s="24" t="n"/>
+      <c r="AJ7" s="33" t="n"/>
+      <c r="AK7" s="33" t="n"/>
+      <c r="AM7" s="33" t="n"/>
+      <c r="AN7" s="33" t="n"/>
+      <c r="AO7" s="33" t="n"/>
+      <c r="AP7" s="33" t="n"/>
+      <c r="AQ7" s="33" t="n"/>
+      <c r="AR7" s="33" t="n"/>
+      <c r="AS7" s="33" t="n"/>
+      <c r="AT7" s="33" t="n"/>
+      <c r="AU7" s="33" t="n"/>
+      <c r="AV7" s="33" t="n"/>
+      <c r="AW7" s="33" t="n"/>
+      <c r="AY7" s="33" t="n"/>
+      <c r="AZ7" s="33" t="n"/>
+      <c r="BA7" s="33" t="n"/>
+      <c r="BB7" s="33" t="n"/>
+      <c r="BC7" s="33" t="n"/>
+      <c r="BD7" s="33" t="n"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1" s="18">
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio Flat / Apart-Hotel</t>
-        </is>
-      </c>
+    <row r="8" ht="15.75" customHeight="1" s="27">
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="33" t="n"/>
+      <c r="J8" s="14" t="n"/>
+      <c r="K8" s="13" t="n"/>
+      <c r="L8" s="13" t="n"/>
+      <c r="N8" s="13" t="n"/>
+      <c r="O8" s="13" t="n"/>
+      <c r="P8" s="13" t="n"/>
+      <c r="Q8" s="13" t="n"/>
+      <c r="R8" s="13" t="n"/>
+      <c r="S8" s="13" t="n"/>
+      <c r="T8" s="13" t="n"/>
+      <c r="U8" s="13" t="n"/>
+      <c r="V8" s="13" t="n"/>
+      <c r="W8" s="13" t="n"/>
+      <c r="X8" s="13" t="n"/>
+      <c r="Y8" s="33" t="n"/>
+      <c r="Z8" s="33" t="n"/>
+      <c r="AA8" s="33" t="n"/>
+      <c r="AB8" s="33" t="n"/>
+      <c r="AC8" s="33" t="n"/>
+      <c r="AD8" s="33" t="n"/>
+      <c r="AE8" s="33" t="n"/>
+      <c r="AF8" s="33" t="n"/>
+      <c r="AG8" s="33" t="n"/>
+      <c r="AH8" s="33" t="n"/>
+      <c r="AI8" s="24" t="n"/>
+      <c r="AJ8" s="33" t="n"/>
+      <c r="AK8" s="33" t="n"/>
+      <c r="AM8" s="33" t="n"/>
+      <c r="AN8" s="33" t="n"/>
+      <c r="AO8" s="33" t="n"/>
+      <c r="AP8" s="33" t="n"/>
+      <c r="AQ8" s="33" t="n"/>
+      <c r="AR8" s="33" t="n"/>
+      <c r="AS8" s="33" t="n"/>
+      <c r="AT8" s="33" t="n"/>
+      <c r="AU8" s="33" t="n"/>
+      <c r="AV8" s="33" t="n"/>
+      <c r="AW8" s="33" t="n"/>
+      <c r="AY8" s="33" t="n"/>
+      <c r="AZ8" s="33" t="n"/>
+      <c r="BA8" s="33" t="n"/>
+      <c r="BB8" s="33" t="n"/>
+      <c r="BC8" s="33" t="n"/>
+      <c r="BD8" s="33" t="n"/>
     </row>
-    <row r="9" ht="14.25" customHeight="1" s="18">
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio Misto - Vertical</t>
-        </is>
-      </c>
+    <row r="9" ht="14.25" customHeight="1" s="27">
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="33" t="n"/>
+      <c r="J9" s="14" t="n"/>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="13" t="n"/>
+      <c r="N9" s="13" t="n"/>
+      <c r="O9" s="13" t="n"/>
+      <c r="P9" s="13" t="n"/>
+      <c r="Q9" s="13" t="n"/>
+      <c r="R9" s="13" t="n"/>
+      <c r="S9" s="13" t="n"/>
+      <c r="T9" s="13" t="n"/>
+      <c r="U9" s="13" t="n"/>
+      <c r="V9" s="13" t="n"/>
+      <c r="W9" s="13" t="n"/>
+      <c r="X9" s="13" t="n"/>
+      <c r="Y9" s="33" t="n"/>
+      <c r="Z9" s="33" t="n"/>
+      <c r="AA9" s="33" t="n"/>
+      <c r="AB9" s="33" t="n"/>
+      <c r="AC9" s="33" t="n"/>
+      <c r="AD9" s="33" t="n"/>
+      <c r="AE9" s="33" t="n"/>
+      <c r="AF9" s="33" t="n"/>
+      <c r="AG9" s="33" t="n"/>
+      <c r="AH9" s="33" t="n"/>
+      <c r="AI9" s="24" t="n"/>
+      <c r="AJ9" s="33" t="n"/>
+      <c r="AK9" s="33" t="n"/>
+      <c r="AM9" s="33" t="n"/>
+      <c r="AN9" s="33" t="n"/>
+      <c r="AO9" s="33" t="n"/>
+      <c r="AP9" s="33" t="n"/>
+      <c r="AQ9" s="33" t="n"/>
+      <c r="AR9" s="33" t="n"/>
+      <c r="AS9" s="33" t="n"/>
+      <c r="AT9" s="33" t="n"/>
+      <c r="AU9" s="33" t="n"/>
+      <c r="AV9" s="33" t="n"/>
+      <c r="AW9" s="33" t="n"/>
+      <c r="AY9" s="33" t="n"/>
+      <c r="AZ9" s="33" t="n"/>
+      <c r="BA9" s="33" t="n"/>
+      <c r="BB9" s="33" t="n"/>
+      <c r="BC9" s="33" t="n"/>
+      <c r="BD9" s="33" t="n"/>
     </row>
-    <row r="10" ht="13.5" customHeight="1" s="18">
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Condomínio Residencial com Comércio no Térreo</t>
-        </is>
-      </c>
+    <row r="10" ht="13.5" customHeight="1" s="27">
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="33" t="n"/>
+      <c r="J10" s="14" t="n"/>
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="13" t="n"/>
+      <c r="N10" s="13" t="n"/>
+      <c r="O10" s="13" t="n"/>
+      <c r="P10" s="13" t="n"/>
+      <c r="Q10" s="13" t="n"/>
+      <c r="R10" s="13" t="n"/>
+      <c r="S10" s="13" t="n"/>
+      <c r="T10" s="13" t="n"/>
+      <c r="U10" s="13" t="n"/>
+      <c r="V10" s="13" t="n"/>
+      <c r="W10" s="13" t="n"/>
+      <c r="X10" s="13" t="n"/>
+      <c r="Y10" s="33" t="n"/>
+      <c r="Z10" s="33" t="n"/>
+      <c r="AA10" s="33" t="n"/>
+      <c r="AB10" s="33" t="n"/>
+      <c r="AC10" s="33" t="n"/>
+      <c r="AD10" s="33" t="n"/>
+      <c r="AE10" s="33" t="n"/>
+      <c r="AF10" s="33" t="n"/>
+      <c r="AG10" s="33" t="n"/>
+      <c r="AH10" s="33" t="n"/>
+      <c r="AI10" s="24" t="n"/>
+      <c r="AJ10" s="33" t="n"/>
+      <c r="AK10" s="33" t="n"/>
+      <c r="AM10" s="33" t="n"/>
+      <c r="AN10" s="33" t="n"/>
+      <c r="AO10" s="33" t="n"/>
+      <c r="AP10" s="33" t="n"/>
+      <c r="AQ10" s="33" t="n"/>
+      <c r="AR10" s="33" t="n"/>
+      <c r="AS10" s="33" t="n"/>
+      <c r="AT10" s="33" t="n"/>
+      <c r="AU10" s="33" t="n"/>
+      <c r="AV10" s="33" t="n"/>
+      <c r="AW10" s="33" t="n"/>
+      <c r="AY10" s="33" t="n"/>
+      <c r="AZ10" s="33" t="n"/>
+      <c r="BA10" s="33" t="n"/>
+      <c r="BB10" s="33" t="n"/>
+      <c r="BC10" s="33" t="n"/>
+      <c r="BD10" s="33" t="n"/>
+    </row>
+    <row r="11">
+      <c r="AA11" s="33" t="n"/>
+      <c r="AB11" s="33" t="n"/>
+      <c r="AC11" s="33" t="n"/>
+      <c r="AD11" s="33" t="n"/>
+      <c r="AE11" s="33" t="n"/>
+      <c r="AF11" s="33" t="n"/>
+      <c r="AG11" s="33" t="n"/>
+      <c r="AH11" s="33" t="n"/>
+      <c r="AI11" s="24" t="n"/>
+      <c r="AJ11" s="33" t="n"/>
+      <c r="AK11" s="33" t="n"/>
+      <c r="AM11" s="33" t="n"/>
+      <c r="AN11" s="33" t="n"/>
+      <c r="AO11" s="33" t="n"/>
+      <c r="AP11" s="33" t="n"/>
+      <c r="AQ11" s="33" t="n"/>
+      <c r="AR11" s="33" t="n"/>
+      <c r="AS11" s="33" t="n"/>
+      <c r="AT11" s="33" t="n"/>
+      <c r="AU11" s="33" t="n"/>
+      <c r="AV11" s="33" t="n"/>
+      <c r="AW11" s="33" t="n"/>
+      <c r="AY11" s="33" t="n"/>
+      <c r="AZ11" s="33" t="n"/>
+      <c r="BA11" s="33" t="n"/>
+      <c r="BB11" s="33" t="n"/>
+      <c r="BC11" s="33" t="n"/>
+      <c r="BD11" s="33" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="T1:X1"/>
-    <mergeCell ref="Y1:AW1"/>
-    <mergeCell ref="AX1:BE1"/>
     <mergeCell ref="N1:R1"/>
+    <mergeCell ref="AW1:BD1"/>
+    <mergeCell ref="Y1:AV1"/>
     <mergeCell ref="B1:C1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="M7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Sim,Não"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
   <pageSetup orientation="portrait" paperSize="9"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;"Aptos"&amp;10 &amp;K000000_x000d_# Interno | Propriedade de Grupo HDI</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10.85546875" bestFit="1" customWidth="1" style="27" min="1" max="1"/>
+    <col width="51.42578125" bestFit="1" customWidth="1" style="27" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" style="27" min="3" max="3"/>
+    <col width="19.7109375" bestFit="1" customWidth="1" style="27" min="4" max="4"/>
+    <col width="43" bestFit="1" customWidth="1" style="27" min="5" max="5"/>
+    <col width="42.140625" bestFit="1" customWidth="1" style="27" min="6" max="6"/>
+    <col width="57.140625" bestFit="1" customWidth="1" style="27" min="7" max="7"/>
+    <col width="31.42578125" bestFit="1" customWidth="1" style="27" min="8" max="8"/>
+    <col width="33.28515625" bestFit="1" customWidth="1" style="27" min="9" max="9"/>
+    <col width="68.140625" bestFit="1" customWidth="1" style="27" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Perfil</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>CBO Tipo de Condomínio</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>CBO Tipo de Construção</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>CBO Objeto Segurado</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>CBO Assistência 24h INPUT</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>O condomínio está legalmente constituído?</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>Deseja contratar indenização a valor de novo? Condominio</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>O Condomínio possui elevador?</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>Qual a quantidade de elevadores?</t>
+        </is>
+      </c>
+      <c r="J1" s="16" t="inlineStr">
+        <is>
+          <t>Período Indenitário" Perda Ou Pagamento de Aluguel a Terceiros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Corretor</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio Comercial - Vertical</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>Superior / Sólida</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>Prédio e Conteúdo</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>Assistência Condomínio Plano Intermediário</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H2" s="22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Operações</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio de Consultórios</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Mista</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>Assistência Condomínio Plano Básico</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="G3" s="21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="H3" s="21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Subscrição</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio de Escritórios</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Não Contratado</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio Exclusivamente Residencial - Horizontal</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio Exclusivamente Residencial - Vertical</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="n"/>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio Flat / Apart-Hotel</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>6 ou mais</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio Misto - Vertical</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Condomínio Residencial com Comércio no Térreo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;"Aptos"&amp;10 &amp;K000000_x000d_# Interno | Propriedade de Grupo HDI</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>